<commit_message>
Plain copy in a personal voice; drop arrows and en dashes
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NtwADbJGLoB7qx1HsTAaRk
</commit_message>
<xml_diff>
--- a/data/kazakhstan-china-trade-2020-2025.xlsx
+++ b/data/kazakhstan-china-trade-2020-2025.xlsx
@@ -434,7 +434,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Kazakhstan's goods trade with China, 2020–2025 ($ billion)</t>
+          <t>Kazakhstan's goods trade with China, 2020-2025 ($ billion)</t>
         </is>
       </c>
     </row>
@@ -468,7 +468,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2020–2021 figures come from news reports citing official bodies and are less reliable than later years.</t>
+          <t>2020-2021 figures come from news reports citing official bodies and are less reliable than later years.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plain copy in a personal voice; drop arrows and en dashes (#4)
Claude-Session: https://claude.ai/code/session_01NtwADbJGLoB7qx1HsTAaRk

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kazakhstan-china-trade-2020-2025.xlsx
+++ b/data/kazakhstan-china-trade-2020-2025.xlsx
@@ -434,7 +434,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Kazakhstan's goods trade with China, 2020–2025 ($ billion)</t>
+          <t>Kazakhstan's goods trade with China, 2020-2025 ($ billion)</t>
         </is>
       </c>
     </row>
@@ -468,7 +468,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2020–2021 figures come from news reports citing official bodies and are less reliable than later years.</t>
+          <t>2020-2021 figures come from news reports citing official bodies and are less reliable than later years.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Trade briefs as statistical bulletins; new brief on China-Russia trade; sector labels
- report(): trade briefs open with a data box and a key-indicators table, numbered sections
- New trade brief: Fewer Cars, Cheaper Oil: China's Trade with Russia, 2020-2025 (GACC data, PDF, XLSX/CSV)
- Kazakhstan-China brief restructured; Chinese series now read directly from the GACC bulletin,
  which corrects 2020-2022 Chinese-data figures (correction noted on the page)
- Company notes show their sector: Banks & fintech, Mining & energy

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kazakhstan-china-trade-2020-2025.xlsx
+++ b/data/kazakhstan-china-trade-2020-2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kazakh data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chinese data" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top products 2024" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="About" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Kazakh data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Chinese data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Top products 2024" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -763,7 +763,7 @@
         <v>13.98</v>
       </c>
       <c r="D3" t="n">
-        <v>16.17</v>
+        <v>16.36</v>
       </c>
       <c r="E3" t="n">
         <v>24.7</v>
@@ -782,22 +782,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>21.5</v>
+        <v>21.45</v>
       </c>
       <c r="C4" t="n">
-        <v>25.2</v>
+        <v>25.25</v>
       </c>
       <c r="D4" t="n">
-        <v>31</v>
+        <v>31.17</v>
       </c>
       <c r="E4" t="n">
-        <v>41</v>
+        <v>41.02</v>
       </c>
       <c r="F4" t="n">
-        <v>43.8</v>
+        <v>43.82</v>
       </c>
       <c r="G4" t="n">
-        <v>48.7</v>
+        <v>48.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
China-Russia trade brief; trade briefs as bulletins; KZ-China correction; sector labels (#9)
* Trade briefs as statistical bulletins; new brief on China-Russia trade; sector labels

- report(): trade briefs open with a data box and a key-indicators table, numbered sections
- New trade brief: Fewer Cars, Cheaper Oil: China's Trade with Russia, 2020-2025 (GACC data, PDF, XLSX/CSV)
- Kazakhstan-China brief restructured; Chinese series now read directly from the GACC bulletin,
  which corrects 2020-2022 Chinese-data figures (correction noted on the page)
- Company notes show their sector: Banks & fintech, Mining & energy

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

* China-Russia brief: add author's comment

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kazakhstan-china-trade-2020-2025.xlsx
+++ b/data/kazakhstan-china-trade-2020-2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kazakh data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chinese data" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top products 2024" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="About" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Kazakh data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Chinese data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Top products 2024" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -763,7 +763,7 @@
         <v>13.98</v>
       </c>
       <c r="D3" t="n">
-        <v>16.17</v>
+        <v>16.36</v>
       </c>
       <c r="E3" t="n">
         <v>24.7</v>
@@ -782,22 +782,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>21.5</v>
+        <v>21.45</v>
       </c>
       <c r="C4" t="n">
-        <v>25.2</v>
+        <v>25.25</v>
       </c>
       <c r="D4" t="n">
-        <v>31</v>
+        <v>31.17</v>
       </c>
       <c r="E4" t="n">
-        <v>41</v>
+        <v>41.02</v>
       </c>
       <c r="F4" t="n">
-        <v>43.8</v>
+        <v>43.82</v>
       </c>
       <c r="G4" t="n">
-        <v>48.7</v>
+        <v>48.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>